<commit_message>
onboarded all devices to 166 server
</commit_message>
<xml_diff>
--- a/things_board/device_data/1334.xlsx
+++ b/things_board/device_data/1334.xlsx
@@ -4807,6 +4807,11 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="7" max="7" width="27.25"/>
+    <col customWidth="1" min="15" max="15" width="16.0"/>
+    <col customWidth="1" min="27" max="27" width="20.0"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -11202,6 +11207,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="7" max="7" width="24.38"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="23" t="s">

</xml_diff>